<commit_message>
Dinesh member changes (pages/excel/core) - base 9f99b6c
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/IP/LSTP_IP_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/IP/LSTP_IP_WF001.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" updateLinks="always"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E166CB-8705-42C0-A9D2-8D79BA31A8B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3FE1AD-190C-4059-8B9C-0C2B5F3429FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TestExecution!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TestExecution!$A$1:$L$1</definedName>
     <definedName name="condition">[1]keywordmapping!$P$22:$P$2000</definedName>
     <definedName name="keywordreqcondition">[1]keywordmapping!$R$2:$R$2000</definedName>
     <definedName name="keywordreqproperty">[1]keywordmapping!$Q$2:$Q$2000</definedName>
@@ -1332,7 +1332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1366,12 +1366,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2733,7 +2732,7 @@
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -2756,7 +2755,7 @@
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -3471,7 +3470,7 @@
       <c r="B69" s="11" t="s">
         <v>376</v>
       </c>
-      <c r="C69" s="25" t="s">
+      <c r="C69" s="24" t="s">
         <v>387</v>
       </c>
       <c r="D69" s="12" t="s">
@@ -3488,7 +3487,7 @@
       <c r="B70" s="11" t="s">
         <v>384</v>
       </c>
-      <c r="C70" s="25" t="s">
+      <c r="C70" s="24" t="s">
         <v>389</v>
       </c>
       <c r="D70" s="11" t="s">
@@ -3505,7 +3504,7 @@
       <c r="B71" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="C71" s="25" t="s">
+      <c r="C71" s="24" t="s">
         <v>389</v>
       </c>
       <c r="F71" s="2" t="s">
@@ -3522,7 +3521,7 @@
       <c r="B72" s="11" t="s">
         <v>379</v>
       </c>
-      <c r="C72" s="25" t="s">
+      <c r="C72" s="24" t="s">
         <v>389</v>
       </c>
       <c r="D72" s="12" t="s">
@@ -3558,17 +3557,17 @@
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="1:11" s="24" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" s="21" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>73</v>
       </c>
-      <c r="B74" s="24" t="s">
+      <c r="B74" s="21" t="s">
         <v>317</v>
       </c>
       <c r="C74" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="F74" s="24" t="s">
+      <c r="F74" s="21" t="s">
         <v>318</v>
       </c>
     </row>
@@ -4983,7 +4982,7 @@
       </c>
     </row>
     <row r="150" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="24"/>
+      <c r="A150" s="21"/>
     </row>
     <row r="151" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B151" s="16" t="s">
@@ -5023,7 +5022,7 @@
       <c r="C154" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:L1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F26 F24 F57 F34 F37 F60 F62 F65 F68 F74 F71" xr:uid="{A78A6BD1-DBA3-4AF4-AD65-FEE2CB211C08}">
       <formula1>IF(ISBLANK(#REF!), INDIRECT("keywordnotreqpage"), IF(ISBLANK(#REF!), INDIRECT("keywordnotreqelement"), INDIRECT(LEFT(#REF!,3)&amp;"")))</formula1>
@@ -5461,4 +5460,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{a4153a30-97aa-49dd-8839-66f72081522c}" enabled="1" method="Standard" siteId="{9ffff5c3-bdfa-4a9d-b595-ff68329945ef}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Excel: banner step-ordering fix (ePMA 27->91, Theatres 26->95 validated); IP + APE workflow edits; batch runner update
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/IP/LSTP_IP_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/IP/LSTP_IP_WF001.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" updateLinks="always" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B9103E2-F1A6-4B4E-BDD8-089568FCCFB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA2C5F5A-B42B-4516-8BF5-F8F488271507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="417">
   <si>
     <t>StepNo</t>
   </si>
@@ -1248,15 +1248,6 @@
     <t>TRANSFER_LOCATION</t>
   </si>
   <si>
-    <t>//Click on Allocate NHS YES</t>
-  </si>
-  <si>
-    <t>//Click on No in Has this person had NHS No pop up</t>
-  </si>
-  <si>
-    <t>//Select finish button PDSSynchronisation</t>
-  </si>
-  <si>
     <t>selectIPHistoryByHeader</t>
   </si>
   <si>
@@ -1299,7 +1290,13 @@
     <t>//validation patient hisotry values</t>
   </si>
   <si>
-    <t>//Select the Appointment details validation from inpatient history</t>
+    <t>Click on Allocate NHS YES</t>
+  </si>
+  <si>
+    <t>Click on No in Has this person had NHS No pop up</t>
+  </si>
+  <si>
+    <t>Select finish button PDSSynchronisation</t>
   </si>
 </sst>
 </file>
@@ -2094,7 +2091,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>19</v>
@@ -2128,7 +2125,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>19</v>
@@ -2574,7 +2571,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>400</v>
+        <v>414</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>69</v>
@@ -2591,7 +2588,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>401</v>
+        <v>415</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>69</v>
@@ -3344,7 +3341,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>312</v>
@@ -3362,22 +3359,22 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D74" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G74" s="3"/>
       <c r="H74" s="3"/>
       <c r="I74" s="22" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="J74" s="3" t="s">
         <v>334</v>
@@ -3957,22 +3954,22 @@
         <v>107</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D108" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E108" s="3"/>
       <c r="F108" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G108" s="3"/>
       <c r="H108" s="3"/>
       <c r="I108" s="22" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="J108" s="3" t="s">
         <v>329</v>
@@ -4031,7 +4028,7 @@
         <v>111</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>402</v>
+        <v>416</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>19</v>
@@ -4744,7 +4741,7 @@
         <v>152</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C153" s="3" t="s">
         <v>312</v>
@@ -4762,22 +4759,22 @@
         <v>153</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C154" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D154" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E154" s="3"/>
       <c r="F154" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G154" s="3"/>
       <c r="H154" s="3"/>
       <c r="I154" s="22" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="J154" s="3" t="s">
         <v>353</v>
@@ -4789,22 +4786,22 @@
         <v>154</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="C155" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D155" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E155" s="3"/>
       <c r="F155" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G155" s="3"/>
       <c r="H155" s="3"/>
       <c r="I155" s="22" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="J155" s="3" t="s">
         <v>356</v>
@@ -4816,25 +4813,25 @@
         <v>155</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="C156" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D156" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E156" s="3"/>
       <c r="F156" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G156" s="3"/>
       <c r="H156" s="3"/>
       <c r="I156" s="22" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="J156" s="3" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="K156" s="24"/>
     </row>
@@ -4906,7 +4903,7 @@
         <v>159</v>
       </c>
       <c r="B160" s="15" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="C160" s="15" t="s">
         <v>312</v>
@@ -4933,25 +4930,25 @@
         <v>160</v>
       </c>
       <c r="B161" s="22" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C161" s="22" t="s">
         <v>312</v>
       </c>
       <c r="D161" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E161" s="22"/>
       <c r="F161" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G161" s="22"/>
       <c r="H161" s="22"/>
       <c r="I161" s="22" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="J161" s="22" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="K161" s="22"/>
     </row>
@@ -5569,7 +5566,7 @@
         <v>196</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C197" s="3" t="s">
         <v>312</v>
@@ -5587,22 +5584,22 @@
         <v>197</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C198" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D198" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E198" s="3"/>
       <c r="F198" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G198" s="3"/>
       <c r="H198" s="3"/>
       <c r="I198" s="22" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="J198" s="3" t="s">
         <v>179</v>
@@ -5818,7 +5815,7 @@
         <v>210</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C211" s="3" t="s">
         <v>312</v>
@@ -5836,22 +5833,22 @@
         <v>211</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="C212" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D212" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E212" s="3"/>
       <c r="F212" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G212" s="3"/>
       <c r="H212" s="3"/>
       <c r="I212" s="22" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="J212" s="3" t="s">
         <v>386</v>
@@ -6084,7 +6081,7 @@
         <v>225</v>
       </c>
       <c r="B226" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C226" s="3" t="s">
         <v>312</v>
@@ -6102,22 +6099,22 @@
         <v>226</v>
       </c>
       <c r="B227" s="3" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="C227" s="3" t="s">
         <v>312</v>
       </c>
       <c r="D227" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E227" s="3"/>
       <c r="F227" s="22" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G227" s="3"/>
       <c r="H227" s="3"/>
       <c r="I227" s="22" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="J227" s="3" t="s">
         <v>207</v>

</xml_diff>